<commit_message>
hab and auto addition
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D148"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4380,6 +4380,682 @@
       </c>
       <c r="D148" t="n">
         <v>80</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>HAB_BR</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>HAB_BR</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>2</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>HAB_LA</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>AS_BR</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>AS_BR</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>2</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>PROGRAM_TR</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>PROGRAM_TR</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>2</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>CBG</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>CBG</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>CPP</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>CPP</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>2</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>YBBG</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>YBBG</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>2</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>YBPP</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>1</v>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>YBPP</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>2</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>PDLD</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>PDLD</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>2</v>
+      </c>
+      <c r="C166" t="n">
+        <v>2</v>
+      </c>
+      <c r="D166" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>LL</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>1</v>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>LL</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>2</v>
+      </c>
+      <c r="C168" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>1</v>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>4</v>
+      </c>
+      <c r="C170" t="n">
+        <v>4</v>
+      </c>
+      <c r="D170" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>DONM</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>1</v>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>ERP</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>2</v>
+      </c>
+      <c r="C172" t="n">
+        <v>2</v>
+      </c>
+      <c r="D172" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>PLUS</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>1</v>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>1</v>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>2</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>CW</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>1</v>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>CW</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>2</v>
+      </c>
+      <c r="C177" t="n">
+        <v>2</v>
+      </c>
+      <c r="D177" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>1</v>
+      </c>
+      <c r="C178" t="n">
+        <v>2</v>
+      </c>
+      <c r="D178" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>3</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>1</v>
+      </c>
+      <c r="C180" t="n">
+        <v>2</v>
+      </c>
+      <c r="D180" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>3</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>LPGE</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>1</v>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>LPGE</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>2</v>
+      </c>
+      <c r="C183" t="n">
+        <v>2</v>
+      </c>
+      <c r="D183" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>AIGO</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>1</v>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>BGL</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>1</v>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>1</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2</v>
+      </c>
+      <c r="C187" t="n">
+        <v>2</v>
+      </c>
+      <c r="D187" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>1</v>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>2</v>
+      </c>
+      <c r="C189" t="n">
+        <v>2</v>
+      </c>
+      <c r="D189" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4393,7 +5069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5060,6 +5736,409 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HAB_BR</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>#,##0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>HAB_LA</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>#,##0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AS_BR</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>#,##0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>YBBG</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>###0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>YBPP</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>###0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PDLD</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LL</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DONM</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DONM</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PLUS</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LPGE</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LPGE</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5071,7 +6150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5529,7 +6608,6 @@
           <t>E:REST</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5560,7 +6638,6 @@
           <t>C:REST</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5591,7 +6668,6 @@
           <t>C:REST</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5617,8 +6693,68 @@
           <t>Entire State</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
all programs ri updates
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D189"/>
+  <dimension ref="A1:D205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5056,6 +5056,270 @@
       </c>
       <c r="D189" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>1</v>
+      </c>
+      <c r="C190" t="n">
+        <v>2</v>
+      </c>
+      <c r="D190" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>3</v>
+      </c>
+      <c r="C191" t="n">
+        <v>3</v>
+      </c>
+      <c r="D191" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>4</v>
+      </c>
+      <c r="C192" t="n">
+        <v>4</v>
+      </c>
+      <c r="D192" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>5</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>1</v>
+      </c>
+      <c r="C194" t="n">
+        <v>2</v>
+      </c>
+      <c r="D194" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>3</v>
+      </c>
+      <c r="C195" t="n">
+        <v>3</v>
+      </c>
+      <c r="D195" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>4</v>
+      </c>
+      <c r="C196" t="n">
+        <v>4</v>
+      </c>
+      <c r="D196" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>5</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>1</v>
+      </c>
+      <c r="C198" t="n">
+        <v>2</v>
+      </c>
+      <c r="D198" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>3</v>
+      </c>
+      <c r="C199" t="n">
+        <v>3</v>
+      </c>
+      <c r="D199" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>4</v>
+      </c>
+      <c r="C200" t="n">
+        <v>4</v>
+      </c>
+      <c r="D200" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>5</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>1</v>
+      </c>
+      <c r="C202" t="n">
+        <v>2</v>
+      </c>
+      <c r="D202" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>3</v>
+      </c>
+      <c r="C203" t="n">
+        <v>3</v>
+      </c>
+      <c r="D203" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>4</v>
+      </c>
+      <c r="C204" t="n">
+        <v>4</v>
+      </c>
+      <c r="D204" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>5</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -5069,7 +5333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6139,6 +6403,90 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>5</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>5</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6150,7 +6498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6751,6 +7099,146 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>B:D</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Amount of Insurance</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>E:REST</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Named Storm Deductible</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NSPPH</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>B:D</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Amount of Insurance</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>E:REST</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Named Storm Deductible</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>B:D</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Amount of Insurance</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>E:REST</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Named Storm Deductible</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NSBGH</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>B:D</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Amount of Insurance</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>E:REST</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Named Storm Deductible</t>
         </is>
       </c>
     </row>
@@ -6818,7 +7306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6852,10 +7340,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>NSPP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fit_width_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NSBG</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fit_width_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>fit_single_page</t>
         </is>

</xml_diff>

<commit_message>
all program and all peril ri updates
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D217"/>
+  <dimension ref="A1:D223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5520,6 +5520,106 @@
       </c>
       <c r="D217" t="n">
         <v>70</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>NSPPP_AP</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>1</v>
+      </c>
+      <c r="C218" t="n">
+        <v>1</v>
+      </c>
+      <c r="D218" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>NSPPP_AP</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>2</v>
+      </c>
+      <c r="C219" t="n">
+        <v>2</v>
+      </c>
+      <c r="D219" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>NSPPP_AP</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>3</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>NSPBG_AP</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>NSPBG_AP</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>2</v>
+      </c>
+      <c r="C222" t="n">
+        <v>2</v>
+      </c>
+      <c r="D222" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>NSPBG_AP</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>3</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
all peril and all program wei changes
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -5633,7 +5633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6782,6 +6782,132 @@
         <v>5</v>
       </c>
       <c r="E54" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>NSPPP</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>NSPPPH</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NSPBG</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>4</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NSPBGH</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NSPPP_AP</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>NSPBG_AP</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>$#,##0</t>
         </is>

</xml_diff>

<commit_message>
formatting of property deductile factor sheets
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -7732,7 +7732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7790,10 +7790,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>PDLD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fit_single_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fit_width_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>fit_single_page</t>
         </is>

</xml_diff>

<commit_message>
formatting of pdf property
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -5687,7 +5687,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
formaating building age modifier
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -7684,7 +7684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7766,10 +7766,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>BABG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fit_width_landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BAPP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>fit_width_landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BABI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fit_width_landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>fit_single_page</t>
         </is>

</xml_diff>

<commit_message>
dollar sign 3 decimel
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -5681,7 +5681,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5765,7 +5765,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5786,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5912,7 +5912,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
state territory multiplier correction
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -7684,7 +7684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7874,10 +7874,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>TRDEF</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fit_single_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>fit_width_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>fit_single_page</t>
         </is>

</xml_diff>

<commit_message>
auto service changes feedback
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -6420,7 +6420,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NoDecimal</t>
+          <t>#,##0</t>
         </is>
       </c>
     </row>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>$#,##0.000</t>
+          <t>$#,##0.00</t>
         </is>
       </c>
     </row>
@@ -6630,7 +6630,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>$#,##0.000</t>
+          <t>$#,##0.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hab formattin for decutible factor
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5572,6 +5572,38 @@
       </c>
       <c r="D220" t="n">
         <v>105</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>PDLD_HAB</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>PDLD_HAB</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>2</v>
+      </c>
+      <c r="C222" t="n">
+        <v>2</v>
+      </c>
+      <c r="D222" t="n">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -5585,7 +5617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6860,6 +6892,27 @@
         <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>PDLD_HAB</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>$#,##0</t>
         </is>

</xml_diff>

<commit_message>
adding service program in bop
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D242"/>
+  <dimension ref="A1:D249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5930,6 +5930,122 @@
       </c>
       <c r="D242" t="n">
         <v>125</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>FU</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>1</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>1</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>1</v>
+      </c>
+      <c r="C245" t="n">
+        <v>3</v>
+      </c>
+      <c r="D245" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>PSS</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>1</v>
+      </c>
+      <c r="C246" t="n">
+        <v>3</v>
+      </c>
+      <c r="D246" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>PSPL</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>1</v>
+      </c>
+      <c r="C247" t="n">
+        <v>1</v>
+      </c>
+      <c r="D247" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>PSPL</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>2</v>
+      </c>
+      <c r="C248" t="n">
+        <v>2</v>
+      </c>
+      <c r="D248" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>MPVS</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>1</v>
+      </c>
+      <c r="C249" t="n">
+        <v>2</v>
+      </c>
+      <c r="D249" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -5943,7 +6059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7409,6 +7525,50 @@
       <c r="E69" t="inlineStr">
         <is>
           <t>#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>FUMP</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>4</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8356,6 @@
           <t>C:REST</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8227,7 +8386,6 @@
           <t>C:REST</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
retail wa 3.c.4.f done
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:D251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6046,6 +6046,38 @@
       </c>
       <c r="D249" t="n">
         <v>150</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>LPGE_RETAIL</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>1</v>
+      </c>
+      <c r="C250" t="n">
+        <v>1</v>
+      </c>
+      <c r="D250" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>LPGE_RETAIL</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>2</v>
+      </c>
+      <c r="C251" t="n">
+        <v>2</v>
+      </c>
+      <c r="D251" t="n">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -6059,7 +6091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7567,6 +7599,48 @@
         <v>4</v>
       </c>
       <c r="E71" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LPGE_RETAIL</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>4</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>LPGE_RETAIL</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" t="n">
+        <v>4</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>$#,##0.00</t>
         </is>

</xml_diff>